<commit_message>
Halloween-Kalkulation: Druckansicht + PDF
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YY7DBkbr5BcFGKyLoSbVN
</commit_message>
<xml_diff>
--- a/drafts/halloween-2026-10-22/kalkulation/Halloween-Kalkulation.xlsx
+++ b/drafts/halloween-2026-10-22/kalkulation/Halloween-Kalkulation.xlsx
@@ -13,6 +13,9 @@
     <sheet name="Warenkorb-Rechnung" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Bestellungen 30 Tage" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">'Bestellungen 30 Tage'!$4:$4</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -23,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="158">
   <si>
     <t xml:space="preserve">Halloween-Aktion: Gewinn mit vs. ohne Aktion</t>
   </si>
@@ -64,25 +67,16 @@
     <t xml:space="preserve">Halloween – gleiche Kunden, gleiche Mengen</t>
   </si>
   <si>
-    <t xml:space="preserve">Halloween – mit Auffüllen (B5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Halloween – mit Auffüllen (B5) und mehr Bestellungen (B6)</t>
+    <t xml:space="preserve">Halloween – mit Auffüllen (gelbes Feld 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Halloween – mit Auffüllen und mehr Bestellungen (gelbe Felder)</t>
   </si>
   <si>
     <t xml:space="preserve">Szenario-Tabelle: Unterschied im Gewinn zu „ohne Aktion“</t>
   </si>
   <si>
-    <t xml:space="preserve">Auffüllen auf 3 Flaschen →</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 %</t>
+    <t xml:space="preserve">Mehr Bestellungen ↓   ·   Anteil, der auf 3 Flaschen auffüllt →</t>
   </si>
   <si>
     <t xml:space="preserve">Anteil auffüllen:</t>
@@ -91,7 +85,7 @@
     <t xml:space="preserve">Break-even</t>
   </si>
   <si>
-    <t xml:space="preserve">Zusätzliche Bestellungen, ab denen sich die Aktion lohnt (ohne Auffüllen)</t>
+    <t xml:space="preserve">Zusätzliche Bestellungen, ab denen sich die Aktion lohnt</t>
   </si>
   <si>
     <t xml:space="preserve">So liest man das</t>
@@ -666,7 +660,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -721,6 +715,10 @@
     </xf>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -1029,7 +1027,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1102,7 +1100,7 @@
         <v>11</v>
       </c>
       <c r="B10" s="7" t="n">
-        <f aca="false">'Bestellungen 30 Tage'!B57*Annahmen!$B$21/Annahmen!$B$20</f>
+        <f aca="false">'Bestellungen 30 Tage'!E57*Annahmen!$B$21/Annahmen!$B$20</f>
         <v>5.525</v>
       </c>
       <c r="C10" s="8" t="n">
@@ -1197,19 +1195,13 @@
       <c r="A16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>19</v>
-      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B17" s="11" t="n">
         <v>0</v>
@@ -1308,12 +1300,12 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>22</v>
+      <c r="A25" s="14" t="s">
+        <v>19</v>
       </c>
       <c r="B25" s="7" t="n">
         <f aca="false">MAX(0,-F11/E11)</f>
@@ -1322,12 +1314,12 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1337,7 +1329,7 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1347,7 +1339,7 @@
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1357,7 +1349,7 @@
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1367,7 +1359,7 @@
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1384,12 +1376,12 @@
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A32:F32"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;A – Seite &amp;P/&amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -1397,7 +1389,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:C21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1409,238 +1401,238 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="B3" s="15" t="n">
         <v>74.9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="B4" s="16" t="n">
         <v>9.5</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="B5" s="17" t="n">
         <v>0.8903</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="B6" s="18" t="n">
         <f aca="false">B4*B5</f>
         <v>8.45785</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="18" t="n">
+        <v>38</v>
+      </c>
+      <c r="B7" s="19" t="n">
         <v>0.2</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B8" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="B8" s="19" t="n">
         <v>0.05</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" s="19" t="n">
+        <v>42</v>
+      </c>
+      <c r="B9" s="20" t="n">
         <v>0.1</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10" s="19" t="n">
+        <v>44</v>
+      </c>
+      <c r="B10" s="20" t="n">
         <v>0.1</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="19" t="n">
+        <v>46</v>
+      </c>
+      <c r="B11" s="20" t="n">
         <v>0.15</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B12" s="19" t="n">
+        <v>47</v>
+      </c>
+      <c r="B12" s="20" t="n">
         <v>0.2</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B13" s="14" t="n">
+        <v>48</v>
+      </c>
+      <c r="B13" s="15" t="n">
         <v>4.9</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B14" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="B14" s="15" t="n">
         <v>150</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="14" t="n">
+        <v>52</v>
+      </c>
+      <c r="B15" s="15" t="n">
         <v>6.19</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B16" s="14" t="n">
+        <v>54</v>
+      </c>
+      <c r="B16" s="15" t="n">
         <v>0.2</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B17" s="14" t="n">
+        <v>56</v>
+      </c>
+      <c r="B17" s="15" t="n">
         <v>4.0346</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B18" s="14" t="n">
+        <v>58</v>
+      </c>
+      <c r="B18" s="15" t="n">
         <v>2.938</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B19" s="17" t="n">
+        <v>60</v>
+      </c>
+      <c r="B19" s="18" t="n">
         <f aca="false">B6</f>
         <v>8.45785</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B20" s="20" t="n">
+        <v>61</v>
+      </c>
+      <c r="B20" s="21" t="n">
         <v>30</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B21" s="21" t="n">
+        <v>63</v>
+      </c>
+      <c r="B21" s="22" t="n">
         <v>3.25</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;A – Seite &amp;P/&amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -1648,7 +1640,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:M35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1661,64 +1653,64 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="K4" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>80</v>
       </c>
       <c r="L4" s="6" t="s">
         <v>8</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5" s="22" t="n">
+        <v>79</v>
+      </c>
+      <c r="B5" s="23" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D5" s="8" t="n">
         <f aca="false">B5*Annahmen!$B$3</f>
@@ -1759,116 +1751,116 @@
       <c r="M5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="B6" s="24" t="n">
+      <c r="A6" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D6" s="25" t="n">
+      <c r="C6" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="26" t="n">
         <f aca="false">B6*Annahmen!$B$3</f>
         <v>74.9</v>
       </c>
-      <c r="E6" s="25" t="n">
+      <c r="E6" s="26" t="n">
         <f aca="false">(B6-INT(B6/3))*Annahmen!$B$3</f>
         <v>74.9</v>
       </c>
-      <c r="F6" s="25" t="n">
+      <c r="F6" s="26" t="n">
         <f aca="false">IF(E6&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>4.9</v>
       </c>
-      <c r="G6" s="25" t="n">
+      <c r="G6" s="26" t="n">
         <f aca="false">E6+F6</f>
         <v>79.8</v>
       </c>
-      <c r="H6" s="25" t="n">
+      <c r="H6" s="26" t="n">
         <f aca="false">B6*Annahmen!$B$6</f>
         <v>8.45785</v>
       </c>
-      <c r="I6" s="25" t="n">
+      <c r="I6" s="26" t="n">
         <f aca="false">IF(E6&gt;=200,Annahmen!$B$17,0)+IF(E6&gt;=350,Annahmen!$B$18,0)+IF(E6&gt;=500,Annahmen!$B$19,0)</f>
         <v>0</v>
       </c>
-      <c r="J6" s="25" t="n">
+      <c r="J6" s="26" t="n">
         <f aca="false">E6*(Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>18.725</v>
       </c>
-      <c r="K6" s="25" t="n">
+      <c r="K6" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L6" s="26" t="n">
+      <c r="L6" s="27" t="n">
         <f aca="false">G6-H6-I6-J6-K6</f>
         <v>46.22715</v>
       </c>
-      <c r="M6" s="25" t="n">
+      <c r="M6" s="26" t="n">
         <f aca="false">L6-L5</f>
         <v>2.24699999999999</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="26" t="n">
         <f aca="false">B7*Annahmen!$B$3</f>
         <v>74.9</v>
       </c>
-      <c r="E7" s="25" t="n">
+      <c r="E7" s="26" t="n">
         <f aca="false">MIN((IF(B7&gt;=10,10*Annahmen!$B$3*(1-Annahmen!$B$12)+(B7-10)*Annahmen!$B$3,IF(B7&gt;=5,5*Annahmen!$B$3*(1-Annahmen!$B$11)+(B7-5)*Annahmen!$B$3,IF(B7&gt;=3,3*Annahmen!$B$3*(1-Annahmen!$B$10)+(B7-3)*Annahmen!$B$3,B7*Annahmen!$B$3))))*(1-Annahmen!$B$9),(B7-INT(B7/3))*Annahmen!$B$3)</f>
         <v>67.41</v>
       </c>
-      <c r="F7" s="25" t="n">
+      <c r="F7" s="26" t="n">
         <f aca="false">IF(E7&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>4.9</v>
       </c>
-      <c r="G7" s="25" t="n">
+      <c r="G7" s="26" t="n">
         <f aca="false">E7+F7</f>
         <v>72.31</v>
       </c>
-      <c r="H7" s="25" t="n">
+      <c r="H7" s="26" t="n">
         <f aca="false">B7*Annahmen!$B$6</f>
         <v>8.45785</v>
       </c>
-      <c r="I7" s="25" t="n">
+      <c r="I7" s="26" t="n">
         <f aca="false">IF(E7&gt;=200,Annahmen!$B$17,0)+IF(E7&gt;=350,Annahmen!$B$18,0)+IF(E7&gt;=500,Annahmen!$B$19,0)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="25" t="n">
+      <c r="J7" s="26" t="n">
         <f aca="false">E7*(Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>16.8525</v>
       </c>
-      <c r="K7" s="25" t="n">
+      <c r="K7" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L7" s="26" t="n">
+      <c r="L7" s="27" t="n">
         <f aca="false">G7-H7-I7-J7-K7</f>
         <v>40.60965</v>
       </c>
-      <c r="M7" s="25" t="n">
+      <c r="M7" s="26" t="n">
         <f aca="false">L7-L5</f>
         <v>-3.37049999999999</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B8" s="22" t="n">
+        <v>79</v>
+      </c>
+      <c r="B8" s="23" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D8" s="8" t="n">
         <f aca="false">B8*Annahmen!$B$3</f>
@@ -1909,116 +1901,116 @@
       <c r="M8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="B9" s="24" t="n">
+      <c r="A9" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D9" s="25" t="n">
+      <c r="C9" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="26" t="n">
         <f aca="false">B9*Annahmen!$B$3</f>
         <v>149.8</v>
       </c>
-      <c r="E9" s="25" t="n">
+      <c r="E9" s="26" t="n">
         <f aca="false">(B9-INT(B9/3))*Annahmen!$B$3</f>
         <v>149.8</v>
       </c>
-      <c r="F9" s="25" t="n">
+      <c r="F9" s="26" t="n">
         <f aca="false">IF(E9&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>4.9</v>
       </c>
-      <c r="G9" s="25" t="n">
+      <c r="G9" s="26" t="n">
         <f aca="false">E9+F9</f>
         <v>154.7</v>
       </c>
-      <c r="H9" s="25" t="n">
+      <c r="H9" s="26" t="n">
         <f aca="false">B9*Annahmen!$B$6</f>
         <v>16.9157</v>
       </c>
-      <c r="I9" s="25" t="n">
+      <c r="I9" s="26" t="n">
         <f aca="false">IF(E9&gt;=200,Annahmen!$B$17,0)+IF(E9&gt;=350,Annahmen!$B$18,0)+IF(E9&gt;=500,Annahmen!$B$19,0)</f>
         <v>0</v>
       </c>
-      <c r="J9" s="25" t="n">
+      <c r="J9" s="26" t="n">
         <f aca="false">E9*(Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>37.45</v>
       </c>
-      <c r="K9" s="25" t="n">
+      <c r="K9" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L9" s="26" t="n">
+      <c r="L9" s="27" t="n">
         <f aca="false">G9-H9-I9-J9-K9</f>
         <v>93.9443</v>
       </c>
-      <c r="M9" s="25" t="n">
+      <c r="M9" s="26" t="n">
         <f aca="false">L9-L8</f>
         <v>4.49400000000001</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B10" s="24" t="n">
-        <v>2</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="D10" s="25" t="n">
+      <c r="D10" s="26" t="n">
         <f aca="false">B10*Annahmen!$B$3</f>
         <v>149.8</v>
       </c>
-      <c r="E10" s="25" t="n">
+      <c r="E10" s="26" t="n">
         <f aca="false">MIN((IF(B10&gt;=10,10*Annahmen!$B$3*(1-Annahmen!$B$12)+(B10-10)*Annahmen!$B$3,IF(B10&gt;=5,5*Annahmen!$B$3*(1-Annahmen!$B$11)+(B10-5)*Annahmen!$B$3,IF(B10&gt;=3,3*Annahmen!$B$3*(1-Annahmen!$B$10)+(B10-3)*Annahmen!$B$3,B10*Annahmen!$B$3))))*(1-Annahmen!$B$9),(B10-INT(B10/3))*Annahmen!$B$3)</f>
         <v>134.82</v>
       </c>
-      <c r="F10" s="25" t="n">
+      <c r="F10" s="26" t="n">
         <f aca="false">IF(E10&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>4.9</v>
       </c>
-      <c r="G10" s="25" t="n">
+      <c r="G10" s="26" t="n">
         <f aca="false">E10+F10</f>
         <v>139.72</v>
       </c>
-      <c r="H10" s="25" t="n">
+      <c r="H10" s="26" t="n">
         <f aca="false">B10*Annahmen!$B$6</f>
         <v>16.9157</v>
       </c>
-      <c r="I10" s="25" t="n">
+      <c r="I10" s="26" t="n">
         <f aca="false">IF(E10&gt;=200,Annahmen!$B$17,0)+IF(E10&gt;=350,Annahmen!$B$18,0)+IF(E10&gt;=500,Annahmen!$B$19,0)</f>
         <v>0</v>
       </c>
-      <c r="J10" s="25" t="n">
+      <c r="J10" s="26" t="n">
         <f aca="false">E10*(Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>33.705</v>
       </c>
-      <c r="K10" s="25" t="n">
+      <c r="K10" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L10" s="26" t="n">
+      <c r="L10" s="27" t="n">
         <f aca="false">G10-H10-I10-J10-K10</f>
         <v>82.7093</v>
       </c>
-      <c r="M10" s="25" t="n">
+      <c r="M10" s="26" t="n">
         <f aca="false">L10-L8</f>
         <v>-6.74099999999999</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B11" s="22" t="n">
+        <v>79</v>
+      </c>
+      <c r="B11" s="23" t="n">
         <v>3</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D11" s="8" t="n">
         <f aca="false">B11*Annahmen!$B$3</f>
@@ -2059,116 +2051,116 @@
       <c r="M11" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="B12" s="24" t="n">
+      <c r="A12" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D12" s="25" t="n">
+      <c r="C12" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="26" t="n">
         <f aca="false">B12*Annahmen!$B$3</f>
         <v>224.7</v>
       </c>
-      <c r="E12" s="25" t="n">
+      <c r="E12" s="26" t="n">
         <f aca="false">(B12-INT(B12/3))*Annahmen!$B$3</f>
         <v>149.8</v>
       </c>
-      <c r="F12" s="25" t="n">
+      <c r="F12" s="26" t="n">
         <f aca="false">IF(E12&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>4.9</v>
       </c>
-      <c r="G12" s="25" t="n">
+      <c r="G12" s="26" t="n">
         <f aca="false">E12+F12</f>
         <v>154.7</v>
       </c>
-      <c r="H12" s="25" t="n">
+      <c r="H12" s="26" t="n">
         <f aca="false">B12*Annahmen!$B$6</f>
         <v>25.37355</v>
       </c>
-      <c r="I12" s="25" t="n">
+      <c r="I12" s="26" t="n">
         <f aca="false">IF(E12&gt;=200,Annahmen!$B$17,0)+IF(E12&gt;=350,Annahmen!$B$18,0)+IF(E12&gt;=500,Annahmen!$B$19,0)</f>
         <v>0</v>
       </c>
-      <c r="J12" s="25" t="n">
+      <c r="J12" s="26" t="n">
         <f aca="false">E12*(Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>37.45</v>
       </c>
-      <c r="K12" s="25" t="n">
+      <c r="K12" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L12" s="26" t="n">
+      <c r="L12" s="27" t="n">
         <f aca="false">G12-H12-I12-J12-K12</f>
         <v>85.48645</v>
       </c>
-      <c r="M12" s="25" t="n">
+      <c r="M12" s="26" t="n">
         <f aca="false">L12-L11</f>
         <v>-28.3556</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B13" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" s="25" t="n">
+      <c r="D13" s="26" t="n">
         <f aca="false">B13*Annahmen!$B$3</f>
         <v>224.7</v>
       </c>
-      <c r="E13" s="25" t="n">
+      <c r="E13" s="26" t="n">
         <f aca="false">MIN((IF(B13&gt;=10,10*Annahmen!$B$3*(1-Annahmen!$B$12)+(B13-10)*Annahmen!$B$3,IF(B13&gt;=5,5*Annahmen!$B$3*(1-Annahmen!$B$11)+(B13-5)*Annahmen!$B$3,IF(B13&gt;=3,3*Annahmen!$B$3*(1-Annahmen!$B$10)+(B13-3)*Annahmen!$B$3,B13*Annahmen!$B$3))))*(1-Annahmen!$B$9),(B13-INT(B13/3))*Annahmen!$B$3)</f>
         <v>149.8</v>
       </c>
-      <c r="F13" s="25" t="n">
+      <c r="F13" s="26" t="n">
         <f aca="false">IF(E13&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>4.9</v>
       </c>
-      <c r="G13" s="25" t="n">
+      <c r="G13" s="26" t="n">
         <f aca="false">E13+F13</f>
         <v>154.7</v>
       </c>
-      <c r="H13" s="25" t="n">
+      <c r="H13" s="26" t="n">
         <f aca="false">B13*Annahmen!$B$6</f>
         <v>25.37355</v>
       </c>
-      <c r="I13" s="25" t="n">
+      <c r="I13" s="26" t="n">
         <f aca="false">IF(E13&gt;=200,Annahmen!$B$17,0)+IF(E13&gt;=350,Annahmen!$B$18,0)+IF(E13&gt;=500,Annahmen!$B$19,0)</f>
         <v>0</v>
       </c>
-      <c r="J13" s="25" t="n">
+      <c r="J13" s="26" t="n">
         <f aca="false">E13*(Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>37.45</v>
       </c>
-      <c r="K13" s="25" t="n">
+      <c r="K13" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L13" s="26" t="n">
+      <c r="L13" s="27" t="n">
         <f aca="false">G13-H13-I13-J13-K13</f>
         <v>85.48645</v>
       </c>
-      <c r="M13" s="25" t="n">
+      <c r="M13" s="26" t="n">
         <f aca="false">L13-L11</f>
         <v>-28.3556</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B14" s="22" t="n">
+        <v>79</v>
+      </c>
+      <c r="B14" s="23" t="n">
         <v>6</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D14" s="8" t="n">
         <f aca="false">B14*Annahmen!$B$3</f>
@@ -2209,116 +2201,116 @@
       <c r="M14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" s="24" t="n">
+      <c r="A15" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="C15" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D15" s="25" t="n">
+      <c r="C15" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="26" t="n">
         <f aca="false">B15*Annahmen!$B$3</f>
         <v>449.4</v>
       </c>
-      <c r="E15" s="25" t="n">
+      <c r="E15" s="26" t="n">
         <f aca="false">(B15-INT(B15/3))*Annahmen!$B$3</f>
         <v>299.6</v>
       </c>
-      <c r="F15" s="25" t="n">
+      <c r="F15" s="26" t="n">
         <f aca="false">IF(E15&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="25" t="n">
+      <c r="G15" s="26" t="n">
         <f aca="false">E15+F15</f>
         <v>299.6</v>
       </c>
-      <c r="H15" s="25" t="n">
+      <c r="H15" s="26" t="n">
         <f aca="false">B15*Annahmen!$B$6</f>
         <v>50.7471</v>
       </c>
-      <c r="I15" s="25" t="n">
+      <c r="I15" s="26" t="n">
         <f aca="false">IF(E15&gt;=200,Annahmen!$B$17,0)+IF(E15&gt;=350,Annahmen!$B$18,0)+IF(E15&gt;=500,Annahmen!$B$19,0)</f>
         <v>4.0346</v>
       </c>
-      <c r="J15" s="25" t="n">
+      <c r="J15" s="26" t="n">
         <f aca="false">E15*(Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>74.9</v>
       </c>
-      <c r="K15" s="25" t="n">
+      <c r="K15" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L15" s="26" t="n">
+      <c r="L15" s="27" t="n">
         <f aca="false">G15-H15-I15-J15-K15</f>
         <v>163.5283</v>
       </c>
-      <c r="M15" s="25" t="n">
+      <c r="M15" s="26" t="n">
         <f aca="false">L15-L14</f>
         <v>-55.484</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="24" t="n">
-        <v>6</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="D16" s="25" t="n">
+      <c r="D16" s="26" t="n">
         <f aca="false">B16*Annahmen!$B$3</f>
         <v>449.4</v>
       </c>
-      <c r="E16" s="25" t="n">
+      <c r="E16" s="26" t="n">
         <f aca="false">MIN((IF(B16&gt;=10,10*Annahmen!$B$3*(1-Annahmen!$B$12)+(B16-10)*Annahmen!$B$3,IF(B16&gt;=5,5*Annahmen!$B$3*(1-Annahmen!$B$11)+(B16-5)*Annahmen!$B$3,IF(B16&gt;=3,3*Annahmen!$B$3*(1-Annahmen!$B$10)+(B16-3)*Annahmen!$B$3,B16*Annahmen!$B$3))))*(1-Annahmen!$B$9),(B16-INT(B16/3))*Annahmen!$B$3)</f>
         <v>299.6</v>
       </c>
-      <c r="F16" s="25" t="n">
+      <c r="F16" s="26" t="n">
         <f aca="false">IF(E16&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="25" t="n">
+      <c r="G16" s="26" t="n">
         <f aca="false">E16+F16</f>
         <v>299.6</v>
       </c>
-      <c r="H16" s="25" t="n">
+      <c r="H16" s="26" t="n">
         <f aca="false">B16*Annahmen!$B$6</f>
         <v>50.7471</v>
       </c>
-      <c r="I16" s="25" t="n">
+      <c r="I16" s="26" t="n">
         <f aca="false">IF(E16&gt;=200,Annahmen!$B$17,0)+IF(E16&gt;=350,Annahmen!$B$18,0)+IF(E16&gt;=500,Annahmen!$B$19,0)</f>
         <v>4.0346</v>
       </c>
-      <c r="J16" s="25" t="n">
+      <c r="J16" s="26" t="n">
         <f aca="false">E16*(Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>74.9</v>
       </c>
-      <c r="K16" s="25" t="n">
+      <c r="K16" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L16" s="26" t="n">
+      <c r="L16" s="27" t="n">
         <f aca="false">G16-H16-I16-J16-K16</f>
         <v>163.5283</v>
       </c>
-      <c r="M16" s="25" t="n">
+      <c r="M16" s="26" t="n">
         <f aca="false">L16-L14</f>
         <v>-55.484</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B17" s="22" t="n">
+        <v>79</v>
+      </c>
+      <c r="B17" s="23" t="n">
         <v>9</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D17" s="8" t="n">
         <f aca="false">B17*Annahmen!$B$3</f>
@@ -2359,116 +2351,116 @@
       <c r="M17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="B18" s="24" t="n">
+      <c r="A18" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B18" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="C18" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D18" s="25" t="n">
+      <c r="C18" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D18" s="26" t="n">
         <f aca="false">B18*Annahmen!$B$3</f>
         <v>674.1</v>
       </c>
-      <c r="E18" s="25" t="n">
+      <c r="E18" s="26" t="n">
         <f aca="false">(B18-INT(B18/3))*Annahmen!$B$3</f>
         <v>449.4</v>
       </c>
-      <c r="F18" s="25" t="n">
+      <c r="F18" s="26" t="n">
         <f aca="false">IF(E18&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>0</v>
       </c>
-      <c r="G18" s="25" t="n">
+      <c r="G18" s="26" t="n">
         <f aca="false">E18+F18</f>
         <v>449.4</v>
       </c>
-      <c r="H18" s="25" t="n">
+      <c r="H18" s="26" t="n">
         <f aca="false">B18*Annahmen!$B$6</f>
         <v>76.12065</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="I18" s="26" t="n">
         <f aca="false">IF(E18&gt;=200,Annahmen!$B$17,0)+IF(E18&gt;=350,Annahmen!$B$18,0)+IF(E18&gt;=500,Annahmen!$B$19,0)</f>
         <v>6.9726</v>
       </c>
-      <c r="J18" s="25" t="n">
+      <c r="J18" s="26" t="n">
         <f aca="false">E18*(Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>112.35</v>
       </c>
-      <c r="K18" s="25" t="n">
+      <c r="K18" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L18" s="26" t="n">
+      <c r="L18" s="27" t="n">
         <f aca="false">G18-H18-I18-J18-K18</f>
         <v>247.56675</v>
       </c>
-      <c r="M18" s="25" t="n">
+      <c r="M18" s="26" t="n">
         <f aca="false">L18-L17</f>
         <v>-99.3981499999999</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="C19" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="24" t="n">
-        <v>9</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="D19" s="25" t="n">
+      <c r="D19" s="26" t="n">
         <f aca="false">B19*Annahmen!$B$3</f>
         <v>674.1</v>
       </c>
-      <c r="E19" s="25" t="n">
+      <c r="E19" s="26" t="n">
         <f aca="false">MIN((IF(B19&gt;=10,10*Annahmen!$B$3*(1-Annahmen!$B$12)+(B19-10)*Annahmen!$B$3,IF(B19&gt;=5,5*Annahmen!$B$3*(1-Annahmen!$B$11)+(B19-5)*Annahmen!$B$3,IF(B19&gt;=3,3*Annahmen!$B$3*(1-Annahmen!$B$10)+(B19-3)*Annahmen!$B$3,B19*Annahmen!$B$3))))*(1-Annahmen!$B$9),(B19-INT(B19/3))*Annahmen!$B$3)</f>
         <v>449.4</v>
       </c>
-      <c r="F19" s="25" t="n">
+      <c r="F19" s="26" t="n">
         <f aca="false">IF(E19&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>0</v>
       </c>
-      <c r="G19" s="25" t="n">
+      <c r="G19" s="26" t="n">
         <f aca="false">E19+F19</f>
         <v>449.4</v>
       </c>
-      <c r="H19" s="25" t="n">
+      <c r="H19" s="26" t="n">
         <f aca="false">B19*Annahmen!$B$6</f>
         <v>76.12065</v>
       </c>
-      <c r="I19" s="25" t="n">
+      <c r="I19" s="26" t="n">
         <f aca="false">IF(E19&gt;=200,Annahmen!$B$17,0)+IF(E19&gt;=350,Annahmen!$B$18,0)+IF(E19&gt;=500,Annahmen!$B$19,0)</f>
         <v>6.9726</v>
       </c>
-      <c r="J19" s="25" t="n">
+      <c r="J19" s="26" t="n">
         <f aca="false">E19*(Annahmen!$B$7+Annahmen!$B$8)</f>
         <v>112.35</v>
       </c>
-      <c r="K19" s="25" t="n">
+      <c r="K19" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L19" s="26" t="n">
+      <c r="L19" s="27" t="n">
         <f aca="false">G19-H19-I19-J19-K19</f>
         <v>247.56675</v>
       </c>
-      <c r="M19" s="25" t="n">
+      <c r="M19" s="26" t="n">
         <f aca="false">L19-L17</f>
         <v>-99.3981499999999</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B20" s="22" t="n">
+        <v>83</v>
+      </c>
+      <c r="B20" s="23" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D20" s="8" t="n">
         <f aca="false">B20*Annahmen!$B$3</f>
@@ -2508,64 +2500,64 @@
       <c r="M20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="B21" s="24" t="n">
+      <c r="A21" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D21" s="25" t="n">
+      <c r="C21" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="26" t="n">
         <f aca="false">B21*Annahmen!$B$3</f>
         <v>74.9</v>
       </c>
-      <c r="E21" s="25" t="n">
+      <c r="E21" s="26" t="n">
         <f aca="false">(B21-INT(B21/3))*Annahmen!$B$3</f>
         <v>74.9</v>
       </c>
-      <c r="F21" s="25" t="n">
+      <c r="F21" s="26" t="n">
         <f aca="false">IF(E21&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>4.9</v>
       </c>
-      <c r="G21" s="25" t="n">
+      <c r="G21" s="26" t="n">
         <f aca="false">E21+F21</f>
         <v>79.8</v>
       </c>
-      <c r="H21" s="25" t="n">
+      <c r="H21" s="26" t="n">
         <f aca="false">B21*Annahmen!$B$6</f>
         <v>8.45785</v>
       </c>
-      <c r="I21" s="25" t="n">
+      <c r="I21" s="26" t="n">
         <f aca="false">IF(E21&gt;=200,Annahmen!$B$17,0)+IF(E21&gt;=350,Annahmen!$B$18,0)+IF(E21&gt;=500,Annahmen!$B$19,0)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="25" t="n">
+      <c r="J21" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L21" s="26" t="n">
+      <c r="L21" s="27" t="n">
         <f aca="false">G21-H21-I21-J21-K21</f>
         <v>64.95215</v>
       </c>
-      <c r="M21" s="25" t="n">
+      <c r="M21" s="26" t="n">
         <f aca="false">L21-L20</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B22" s="22" t="n">
+        <v>83</v>
+      </c>
+      <c r="B22" s="23" t="n">
         <v>2</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D22" s="8" t="n">
         <f aca="false">B22*Annahmen!$B$3</f>
@@ -2605,64 +2597,64 @@
       <c r="M22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="B23" s="24" t="n">
+      <c r="A23" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B23" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="C23" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D23" s="25" t="n">
+      <c r="C23" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" s="26" t="n">
         <f aca="false">B23*Annahmen!$B$3</f>
         <v>149.8</v>
       </c>
-      <c r="E23" s="25" t="n">
+      <c r="E23" s="26" t="n">
         <f aca="false">(B23-INT(B23/3))*Annahmen!$B$3</f>
         <v>149.8</v>
       </c>
-      <c r="F23" s="25" t="n">
+      <c r="F23" s="26" t="n">
         <f aca="false">IF(E23&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>4.9</v>
       </c>
-      <c r="G23" s="25" t="n">
+      <c r="G23" s="26" t="n">
         <f aca="false">E23+F23</f>
         <v>154.7</v>
       </c>
-      <c r="H23" s="25" t="n">
+      <c r="H23" s="26" t="n">
         <f aca="false">B23*Annahmen!$B$6</f>
         <v>16.9157</v>
       </c>
-      <c r="I23" s="25" t="n">
+      <c r="I23" s="26" t="n">
         <f aca="false">IF(E23&gt;=200,Annahmen!$B$17,0)+IF(E23&gt;=350,Annahmen!$B$18,0)+IF(E23&gt;=500,Annahmen!$B$19,0)</f>
         <v>0</v>
       </c>
-      <c r="J23" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="25" t="n">
+      <c r="J23" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L23" s="26" t="n">
+      <c r="L23" s="27" t="n">
         <f aca="false">G23-H23-I23-J23-K23</f>
         <v>131.3943</v>
       </c>
-      <c r="M23" s="25" t="n">
+      <c r="M23" s="26" t="n">
         <f aca="false">L23-L22</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B24" s="22" t="n">
+        <v>83</v>
+      </c>
+      <c r="B24" s="23" t="n">
         <v>3</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D24" s="8" t="n">
         <f aca="false">B24*Annahmen!$B$3</f>
@@ -2702,64 +2694,64 @@
       <c r="M24" s="8"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="B25" s="24" t="n">
+      <c r="A25" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B25" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="C25" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D25" s="25" t="n">
+      <c r="C25" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D25" s="26" t="n">
         <f aca="false">B25*Annahmen!$B$3</f>
         <v>224.7</v>
       </c>
-      <c r="E25" s="25" t="n">
+      <c r="E25" s="26" t="n">
         <f aca="false">(B25-INT(B25/3))*Annahmen!$B$3</f>
         <v>149.8</v>
       </c>
-      <c r="F25" s="25" t="n">
+      <c r="F25" s="26" t="n">
         <f aca="false">IF(E25&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>4.9</v>
       </c>
-      <c r="G25" s="25" t="n">
+      <c r="G25" s="26" t="n">
         <f aca="false">E25+F25</f>
         <v>154.7</v>
       </c>
-      <c r="H25" s="25" t="n">
+      <c r="H25" s="26" t="n">
         <f aca="false">B25*Annahmen!$B$6</f>
         <v>25.37355</v>
       </c>
-      <c r="I25" s="25" t="n">
+      <c r="I25" s="26" t="n">
         <f aca="false">IF(E25&gt;=200,Annahmen!$B$17,0)+IF(E25&gt;=350,Annahmen!$B$18,0)+IF(E25&gt;=500,Annahmen!$B$19,0)</f>
         <v>0</v>
       </c>
-      <c r="J25" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="25" t="n">
+      <c r="J25" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L25" s="26" t="n">
+      <c r="L25" s="27" t="n">
         <f aca="false">G25-H25-I25-J25-K25</f>
         <v>122.93645</v>
       </c>
-      <c r="M25" s="25" t="n">
+      <c r="M25" s="26" t="n">
         <f aca="false">L25-L24</f>
         <v>-43.4954</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B26" s="22" t="n">
+        <v>83</v>
+      </c>
+      <c r="B26" s="23" t="n">
         <v>6</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D26" s="8" t="n">
         <f aca="false">B26*Annahmen!$B$3</f>
@@ -2799,64 +2791,64 @@
       <c r="M26" s="8"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="B27" s="24" t="n">
+      <c r="A27" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B27" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="C27" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D27" s="25" t="n">
+      <c r="C27" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D27" s="26" t="n">
         <f aca="false">B27*Annahmen!$B$3</f>
         <v>449.4</v>
       </c>
-      <c r="E27" s="25" t="n">
+      <c r="E27" s="26" t="n">
         <f aca="false">(B27-INT(B27/3))*Annahmen!$B$3</f>
         <v>299.6</v>
       </c>
-      <c r="F27" s="25" t="n">
+      <c r="F27" s="26" t="n">
         <f aca="false">IF(E27&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="25" t="n">
+      <c r="G27" s="26" t="n">
         <f aca="false">E27+F27</f>
         <v>299.6</v>
       </c>
-      <c r="H27" s="25" t="n">
+      <c r="H27" s="26" t="n">
         <f aca="false">B27*Annahmen!$B$6</f>
         <v>50.7471</v>
       </c>
-      <c r="I27" s="25" t="n">
+      <c r="I27" s="26" t="n">
         <f aca="false">IF(E27&gt;=200,Annahmen!$B$17,0)+IF(E27&gt;=350,Annahmen!$B$18,0)+IF(E27&gt;=500,Annahmen!$B$19,0)</f>
         <v>4.0346</v>
       </c>
-      <c r="J27" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="25" t="n">
+      <c r="J27" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L27" s="26" t="n">
+      <c r="L27" s="27" t="n">
         <f aca="false">G27-H27-I27-J27-K27</f>
         <v>238.4283</v>
       </c>
-      <c r="M27" s="25" t="n">
+      <c r="M27" s="26" t="n">
         <f aca="false">L27-L26</f>
         <v>-90.687</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B28" s="22" t="n">
+        <v>83</v>
+      </c>
+      <c r="B28" s="23" t="n">
         <v>9</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D28" s="8" t="n">
         <f aca="false">B28*Annahmen!$B$3</f>
@@ -2896,87 +2888,87 @@
       <c r="M28" s="8"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="B29" s="24" t="n">
+      <c r="A29" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B29" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="C29" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="D29" s="25" t="n">
+      <c r="C29" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D29" s="26" t="n">
         <f aca="false">B29*Annahmen!$B$3</f>
         <v>674.1</v>
       </c>
-      <c r="E29" s="25" t="n">
+      <c r="E29" s="26" t="n">
         <f aca="false">(B29-INT(B29/3))*Annahmen!$B$3</f>
         <v>449.4</v>
       </c>
-      <c r="F29" s="25" t="n">
+      <c r="F29" s="26" t="n">
         <f aca="false">IF(E29&gt;=Annahmen!$B$14,0,Annahmen!$B$13)</f>
         <v>0</v>
       </c>
-      <c r="G29" s="25" t="n">
+      <c r="G29" s="26" t="n">
         <f aca="false">E29+F29</f>
         <v>449.4</v>
       </c>
-      <c r="H29" s="25" t="n">
+      <c r="H29" s="26" t="n">
         <f aca="false">B29*Annahmen!$B$6</f>
         <v>76.12065</v>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="I29" s="26" t="n">
         <f aca="false">IF(E29&gt;=200,Annahmen!$B$17,0)+IF(E29&gt;=350,Annahmen!$B$18,0)+IF(E29&gt;=500,Annahmen!$B$19,0)</f>
         <v>6.9726</v>
       </c>
-      <c r="J29" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" s="25" t="n">
+      <c r="J29" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="26" t="n">
         <f aca="false">Annahmen!$B$15+Annahmen!$B$16</f>
         <v>6.39</v>
       </c>
-      <c r="L29" s="26" t="n">
+      <c r="L29" s="27" t="n">
         <f aca="false">G29-H29-I29-J29-K29</f>
         <v>359.91675</v>
       </c>
-      <c r="M29" s="25" t="n">
+      <c r="M29" s="26" t="n">
         <f aca="false">L29-L28</f>
         <v>-160.06715</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;A – Seite &amp;P/&amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -2984,7 +2976,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:J60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2999,52 +2991,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>1</v>
@@ -3073,10 +3065,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>1</v>
@@ -3105,10 +3097,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>0</v>
@@ -3137,10 +3129,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>0</v>
@@ -3169,10 +3161,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>1</v>
@@ -3201,10 +3193,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>0</v>
@@ -3233,10 +3225,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>1</v>
@@ -3265,10 +3257,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>2</v>
@@ -3297,10 +3289,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C13" s="4" t="n">
         <v>3</v>
@@ -3329,10 +3321,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C14" s="4" t="n">
         <v>1</v>
@@ -3361,10 +3353,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C15" s="4" t="n">
         <v>1</v>
@@ -3393,10 +3385,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C16" s="4" t="n">
         <v>1</v>
@@ -3425,10 +3417,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C17" s="4" t="n">
         <v>0</v>
@@ -3457,10 +3449,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>1</v>
@@ -3489,10 +3481,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C19" s="4" t="n">
         <v>2</v>
@@ -3521,10 +3513,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>1</v>
@@ -3553,10 +3545,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>1</v>
@@ -3585,10 +3577,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C22" s="4" t="n">
         <v>0</v>
@@ -3617,10 +3609,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C23" s="4" t="n">
         <v>0</v>
@@ -3649,10 +3641,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C24" s="4" t="n">
         <v>0</v>
@@ -3681,10 +3673,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C25" s="4" t="n">
         <v>1</v>
@@ -3713,10 +3705,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C26" s="4" t="n">
         <v>1</v>
@@ -3745,10 +3737,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C27" s="4" t="n">
         <v>0</v>
@@ -3777,10 +3769,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C28" s="4" t="n">
         <v>1</v>
@@ -3809,10 +3801,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C29" s="4" t="n">
         <v>2</v>
@@ -3841,10 +3833,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C30" s="4" t="n">
         <v>0</v>
@@ -3873,10 +3865,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C31" s="4" t="n">
         <v>1</v>
@@ -3905,10 +3897,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C32" s="4" t="n">
         <v>0</v>
@@ -3937,10 +3929,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C33" s="4" t="n">
         <v>0</v>
@@ -3969,10 +3961,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C34" s="4" t="n">
         <v>2</v>
@@ -4001,10 +3993,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C35" s="4" t="n">
         <v>0</v>
@@ -4033,10 +4025,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C36" s="4" t="n">
         <v>3</v>
@@ -4065,10 +4057,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C37" s="4" t="n">
         <v>1</v>
@@ -4097,10 +4089,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C38" s="4" t="n">
         <v>3</v>
@@ -4129,10 +4121,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C39" s="4" t="n">
         <v>1</v>
@@ -4161,10 +4153,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C40" s="4" t="n">
         <v>1</v>
@@ -4193,10 +4185,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C41" s="4" t="n">
         <v>2</v>
@@ -4225,10 +4217,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C42" s="4" t="n">
         <v>1</v>
@@ -4257,10 +4249,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C43" s="4" t="n">
         <v>1</v>
@@ -4289,10 +4281,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C44" s="4" t="n">
         <v>2</v>
@@ -4321,10 +4313,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C45" s="4" t="n">
         <v>1</v>
@@ -4353,10 +4345,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C46" s="4" t="n">
         <v>3</v>
@@ -4385,10 +4377,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C47" s="4" t="n">
         <v>1</v>
@@ -4417,10 +4409,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C48" s="4" t="n">
         <v>0</v>
@@ -4449,10 +4441,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C49" s="4" t="n">
         <v>1</v>
@@ -4481,10 +4473,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C50" s="4" t="n">
         <v>1</v>
@@ -4513,10 +4505,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C51" s="4" t="n">
         <v>0</v>
@@ -4545,10 +4537,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C52" s="4" t="n">
         <v>0</v>
@@ -4577,10 +4569,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C53" s="4" t="n">
         <v>0</v>
@@ -4609,10 +4601,10 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C54" s="4" t="n">
         <v>3</v>
@@ -4641,10 +4633,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C55" s="4" t="n">
         <v>1</v>
@@ -4673,7 +4665,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C56" s="3" t="n">
         <f aca="false">SUM(C5:C55)</f>
@@ -4710,43 +4702,43 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="B57" s="4" t="n">
+        <v>154</v>
+      </c>
+      <c r="E57" s="4" t="n">
         <f aca="false">COUNTA(A5:A55)</f>
         <v>51</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="B58" s="4" t="n">
+        <v>155</v>
+      </c>
+      <c r="E58" s="4" t="n">
         <f aca="false">COUNTIF(B5:B55,"Ja")</f>
         <v>36</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B59" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="E59" s="4" t="n">
         <f aca="false">SUMPRODUCT((G5:G55&gt;E5:E55+0.05)*1)</f>
         <v>25</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="27" t="s">
-        <v>160</v>
+      <c r="A60" s="28" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;A – Seite &amp;P/&amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>